<commit_message>
map more cm columns for cells
</commit_message>
<xml_diff>
--- a/backend/templates/template_cell_3g.xlsx
+++ b/backend/templates/template_cell_3g.xlsx
@@ -37872,7 +37872,7 @@
       <formula2>30</formula2>
     </dataValidation>
     <dataValidation sqref="S2:S1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
-      <formula1>'_Lookups'!$C$2:$C$68</formula1>
+      <formula1>'_Lookups'!$C$2:$C$83</formula1>
     </dataValidation>
     <dataValidation sqref="W2:W1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"2x2,4x4,8x8"</formula1>
@@ -39236,7 +39236,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GRENTECH|SGR-DTX-YC-18</t>
+          <t>ERICSSON|AIR3219B77U</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -39258,7 +39258,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>HENGXIN|HX4W3319B2RNF</t>
+          <t>ERICSSON|AIR3265B41</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -39280,7 +39280,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>HENGXIN|HXHH3820B2-EU</t>
+          <t>ERICSSON|AIR6419B41</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -39302,7 +39302,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>HUAWEI|A19451811V01</t>
+          <t>ERICSSON|AIR6419B77D</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -39324,7 +39324,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>HUAWEI|A19451811V06</t>
+          <t>GRENTECH|SGR-DTX-YC-18</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -39346,7 +39346,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hengxin|HX4W6518DEF</t>
+          <t>HENGXIN|HX4W3319B2RNF</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -39368,7 +39368,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>KATHREIN|739623</t>
+          <t>HENGXIN|HXHH3820B2-EU</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -39390,7 +39390,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>KATHREIN|741 785</t>
+          <t>HUAWEI|A04040PA00v06</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -39412,7 +39412,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>KATHREIN|741322</t>
+          <t>HUAWEI|A19451811V01</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -39434,7 +39434,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>KATHREIN|742215</t>
+          <t>HUAWEI|A19451811V06</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -39456,7 +39456,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>KATHREIN|742222V01</t>
+          <t>HUAWEI|AAU5336v</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -39478,7 +39478,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>KATHREIN|742266V02</t>
+          <t>HUAWEI|AAU5356</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -39500,7 +39500,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>KATHREIN|800 10492V01</t>
+          <t>HUAWEI|AAU5636m</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -39522,7 +39522,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>KATHREIN|80010428</t>
+          <t>HUAWEI|AAU5636v</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -39544,7 +39544,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MOBI|MB3F-65-18DE10</t>
+          <t>HUAWEI|ADU4517R51v06</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -39566,7 +39566,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MOBI|MB900/1800-65-17/18DE10/8-C-VN</t>
+          <t>HUAWEI|AMB4519R47v06</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -39588,7 +39588,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NETOP|S-WAVE U-65-12D</t>
+          <t>Hengxin|HX4W6518DEF</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -39605,7 +39605,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>POWERSTORM|C-BXH-65606580-M</t>
+          <t>KATHREIN|739623</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -39622,7 +39622,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PROSE|2G4W4XBF-27</t>
+          <t>KATHREIN|741 785</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -39639,7 +39639,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PROSE|S-WAVE EW_EW-65-14D-64F-O1</t>
+          <t>KATHREIN|741322</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -39656,7 +39656,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>RFS|APX-906516L-0T0</t>
+          <t>KATHREIN|742215</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -39673,7 +39673,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>RFS|APX86-906516L-T6</t>
+          <t>KATHREIN|742222V01</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -39690,7 +39690,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>RFS|APXE20F-T6</t>
+          <t>KATHREIN|742266V02</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -39707,7 +39707,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ROSENBERGER|4WC-11M</t>
+          <t>KATHREIN|800 10492V01</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -39724,7 +39724,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ROSENBERGER|CA-D3W5V32F-SD01</t>
+          <t>KATHREIN|80010428</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -39741,7 +39741,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ROSENBERGER|G3WF-11M</t>
+          <t>MOBI|MB3F-65-18DE10</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -39758,7 +39758,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE 0809/U-65-18DV8</t>
+          <t>MOBI|MB900/1800-65-17/18DE10/8-C-VN</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -39775,7 +39775,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE 0809/U/U-65-18DV8-B5</t>
+          <t>NETOP|S-WAVE U-65-12D</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -39792,7 +39792,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE 09-65-18DV10-B3</t>
+          <t>NOKIA|AQHC</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -39809,7 +39809,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE 1800-65-18DT6</t>
+          <t>NOKIA|AQQV</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -39826,7 +39826,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE 7FW-10/12-LP</t>
+          <t>NOKIA|AVHA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -39843,7 +39843,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE 7FW-180-4/4.5-O2</t>
+          <t>NOKIA|AVQG</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -39860,7 +39860,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE 7FW-OD-3-L500</t>
+          <t>POWERSTORM|C-BXH-65606580-M</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -39877,7 +39877,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE EW/EW-65-14D-O1</t>
+          <t>PROSE|2G4W4XBF-27</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -39894,7 +39894,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE EW/EW-65-18DV2/12-VN1</t>
+          <t>PROSE|S-WAVE EW_EW-65-14D-64F-O1</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -39911,7 +39911,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE EW/EW-65-9D-O1</t>
+          <t>RFS|APX-906516L-0T0</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -39928,7 +39928,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE U-33-20DV10</t>
+          <t>RFS|APX86-906516L-T6</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -39945,7 +39945,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE U-65-18DV10-B4</t>
+          <t>RFS|APXE20F-T6</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -39962,7 +39962,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE U/U-33-20DV10-BS</t>
+          <t>ROSENBERGER|4WC-11M</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -39979,7 +39979,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ROSENBERGER|S-WAVE U/U/U-33-21DT6-TS</t>
+          <t>ROSENBERGER|CA-D3W5V32F-SD01</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -39996,7 +39996,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>TONGYU|T0004M3V011</t>
+          <t>ROSENBERGER|G3WF-11M</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -40013,7 +40013,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>TONGYU|TDJ-809018DM-65FT0</t>
+          <t>ROSENBERGER|S-WAVE 0809/U-65-18DV8</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -40030,7 +40030,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>TONGYU|TDJ-9018/1818DM-65PT6-C</t>
+          <t>ROSENBERGER|S-WAVE 0809/U/U-65-18DV8-B5</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -40047,7 +40047,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>TONGYU|TDJ-9018DM-65FT0</t>
+          <t>ROSENBERGER|S-WAVE 09-65-18DV10-B3</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -40064,7 +40064,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>TONGYU|TDJH-182018DE-65F</t>
+          <t>ROSENBERGER|S-WAVE 1800-65-18DT6</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -40081,7 +40081,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>TONGYU|TDQ-172722DEI-33FT2V3</t>
+          <t>ROSENBERGER|S-WAVE 7FW-10/12-LP</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -40098,7 +40098,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>YOLYCOM|YLPXT3S17216518-6MP</t>
+          <t>ROSENBERGER|S-WAVE 7FW-180-4/4.5-O2</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -40115,7 +40115,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>ROSENBERGER|S-WAVE 7FW-OD-3-L500</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -40132,7 +40132,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>test1</t>
+          <t>ROSENBERGER|S-WAVE EW/EW-65-14D-O1</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -40149,7 +40149,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>test2</t>
+          <t>ROSENBERGER|S-WAVE EW/EW-65-18DV2/12-VN1</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -40164,6 +40164,11 @@
           <t>Phường Bình Khê</t>
         </is>
       </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>ROSENBERGER|S-WAVE EW/EW-65-9D-O1</t>
+        </is>
+      </c>
       <c r="D69" t="inlineStr">
         <is>
           <t>RSGTB2E</t>
@@ -40176,6 +40181,11 @@
           <t>Phường Bình Kiến</t>
         </is>
       </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>ROSENBERGER|S-WAVE U-33-20DV10</t>
+        </is>
+      </c>
       <c r="D70" t="inlineStr">
         <is>
           <t>RTGMT3N</t>
@@ -40188,6 +40198,11 @@
           <t>Phường Bình Long</t>
         </is>
       </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>ROSENBERGER|S-WAVE U-65-18DV10-B4</t>
+        </is>
+      </c>
       <c r="D71" t="inlineStr">
         <is>
           <t>iHNCG1H</t>
@@ -40200,6 +40215,11 @@
           <t>Phường Bình Lộc</t>
         </is>
       </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ROSENBERGER|S-WAVE U/U-33-20DV10-BS</t>
+        </is>
+      </c>
       <c r="D72" t="inlineStr">
         <is>
           <t>iHNCG3H</t>
@@ -40212,6 +40232,11 @@
           <t>Phường Bình Lợi Trung</t>
         </is>
       </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ROSENBERGER|S-WAVE U/U/U-33-21DT6-TS</t>
+        </is>
+      </c>
       <c r="D73" t="inlineStr">
         <is>
           <t>iHNHM1H</t>
@@ -40224,6 +40249,11 @@
           <t>Phường Bình Minh</t>
         </is>
       </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>TONGYU|T0004M3V011</t>
+        </is>
+      </c>
       <c r="D74" t="inlineStr">
         <is>
           <t>iHNHM2H</t>
@@ -40236,6 +40266,11 @@
           <t>Phường Bình Phú</t>
         </is>
       </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>TONGYU|TDJ-809018DM-65FT0</t>
+        </is>
+      </c>
       <c r="D75" t="inlineStr">
         <is>
           <t>iHNHM3H</t>
@@ -40248,6 +40283,11 @@
           <t>Phường Bình Phước</t>
         </is>
       </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>TONGYU|TDJ-9018/1818DM-65PT6-C</t>
+        </is>
+      </c>
       <c r="D76" t="inlineStr">
         <is>
           <t>iHNHM5H</t>
@@ -40260,6 +40300,11 @@
           <t>Phường Bình Quới</t>
         </is>
       </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>TONGYU|TDJ-9018DM-65FT0</t>
+        </is>
+      </c>
       <c r="D77" t="inlineStr">
         <is>
           <t>iHNHM6H</t>
@@ -40272,6 +40317,11 @@
           <t>Phường Bình Thuận</t>
         </is>
       </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>TONGYU|TDJH-182018DE-65F</t>
+        </is>
+      </c>
       <c r="D78" t="inlineStr">
         <is>
           <t>iHNHM7H</t>
@@ -40284,6 +40334,11 @@
           <t>Phường Bình Thạnh</t>
         </is>
       </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>TONGYU|TDQ-172722DEI-33FT2V3</t>
+        </is>
+      </c>
       <c r="D79" t="inlineStr">
         <is>
           <t>iHNHM8H</t>
@@ -40296,6 +40351,11 @@
           <t>Phường Bình Thới</t>
         </is>
       </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>YOLYCOM|YLPXT3S17216518-6MP</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="B81" t="inlineStr">
@@ -40303,6 +40363,11 @@
           <t>Phường Bình Thủy</t>
         </is>
       </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
@@ -40310,11 +40375,21 @@
           <t>Phường Bình Tiên</t>
         </is>
       </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
           <t>Phường Bình Trưng</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>test2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add IBC value type for sites and cells
</commit_message>
<xml_diff>
--- a/backend/templates/template_cell_3g.xlsx
+++ b/backend/templates/template_cell_3g.xlsx
@@ -37821,7 +37821,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AI1"/>
-  <dataValidations count="20">
+  <dataValidations count="15">
     <dataValidation sqref="A2:A1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"MB,MT,MN"</formula1>
     </dataValidation>
@@ -37850,26 +37850,6 @@
     </dataValidation>
     <dataValidation sqref="M2:M1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>"Ericsson,Nokia,Huawei,ZTE,Samsung"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Độ cao không hợp lệ" error="Phải là số dương (m)" type="decimal" operator="between">
-      <formula1>0</formula1>
-      <formula2>999</formula2>
-    </dataValidation>
-    <dataValidation sqref="O2:O1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Azimuth không hợp lệ" error="Azimuth phải trong khoảng 0–359" type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>359</formula2>
-    </dataValidation>
-    <dataValidation sqref="P2:P1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="M-tilt không hợp lệ" error="M-tilt thường trong khoảng -30 đến 30" type="decimal" operator="between">
-      <formula1>-30</formula1>
-      <formula2>30</formula2>
-    </dataValidation>
-    <dataValidation sqref="Q2:Q1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="E-Tilt không hợp lệ" error="E-Tilt thường trong khoảng -30 đến 30" type="decimal" operator="between">
-      <formula1>-30</formula1>
-      <formula2>30</formula2>
-    </dataValidation>
-    <dataValidation sqref="R2:R1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Total Tilt không hợp lệ" error="Total Tilt thường trong khoảng -30 đến 30" type="decimal" operator="between">
-      <formula1>-30</formula1>
-      <formula2>30</formula2>
     </dataValidation>
     <dataValidation sqref="S2:S1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách" type="list">
       <formula1>'_Lookups'!$C$2:$C$83</formula1>
@@ -38440,7 +38420,7 @@
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>Độ cao anten (m) – bắt buộc, số dương</t>
+          <t>Độ cao anten – bắt buộc (số hoặc chuỗi, vd: 28 hoặc IBC)</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
@@ -38457,7 +38437,7 @@
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>Góc phương vị – bắt buộc, trong 0–359</t>
+          <t>Góc phương vị – bắt buộc (số hoặc chuỗi, vd: 120 hoặc IBC)</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
@@ -38474,7 +38454,7 @@
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>Mechanical tilt – bắt buộc</t>
+          <t>Mechanical tilt – bắt buộc (số hoặc chuỗi, vd: 2 hoặc IBC)</t>
         </is>
       </c>
       <c r="C45" s="15" t="inlineStr">
@@ -38491,7 +38471,7 @@
       </c>
       <c r="B46" s="13" t="inlineStr">
         <is>
-          <t>Electrical tilt – bắt buộc</t>
+          <t>Electrical tilt – bắt buộc (số hoặc chuỗi, vd: 4 hoặc IBC)</t>
         </is>
       </c>
       <c r="C46" s="15" t="inlineStr">
@@ -38508,7 +38488,7 @@
       </c>
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>Tổng tilt = M-tilt + E-Tilt (tự tính hoặc để trống)</t>
+          <t>Tổng tilt (số hoặc chuỗi, tự tính hoặc để trống)</t>
         </is>
       </c>
       <c r="C47" s="14" t="inlineStr">

</xml_diff>